<commit_message>
#22 Speaker part added in Client and eSpark BOM
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Speaker-v1.2/BOM/Client BOM IoT-Speaker.xlsx
+++ b/Design Files/IoT-Speaker-v1.2/BOM/Client BOM IoT-Speaker.xlsx
@@ -5,21 +5,22 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Speaker-v1.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="2 Boards" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="278">
   <si>
     <t>Component list</t>
   </si>
@@ -840,10 +841,19 @@
     <t>Adaptor</t>
   </si>
   <si>
-    <t>Universal 5V 1A 2A Type C USB Charger Mobile Phone Wall Travel Power Adapter Charger EU/US Plug For Huawei Xiaomi iPhone Samsung</t>
-  </si>
-  <si>
     <t>DNP</t>
+  </si>
+  <si>
+    <t>Universal 5V 1A 2A Type C USB Charger Mobile Phone Wall Travel Power Adapter Charger EU/US Plug For Huawei Xiaomi iPhone Samsung ( 2A Rating Selected)</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>FS40DS0430-H18.8</t>
+  </si>
+  <si>
+    <t>Speakers ROHS</t>
   </si>
 </sst>
 </file>
@@ -853,7 +863,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1013,6 +1023,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1257,7 +1274,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1417,6 +1434,21 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1426,14 +1458,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1501,6 +1530,60 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="20059650" y="629542"/>
+          <a:ext cx="1857375" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>19942</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1905000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14668500" y="629542"/>
           <a:ext cx="1857375" cy="1104008"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1777,7 +1860,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1803,11 +1886,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1845,7 +1928,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="61"/>
+      <c r="M3" s="66"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1864,7 +1947,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="62"/>
+      <c r="M4" s="67"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1883,7 +1966,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="62"/>
+      <c r="M5" s="67"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1898,7 +1981,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="62"/>
+      <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1913,7 +1996,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="62"/>
+      <c r="M7" s="67"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1928,7 +2011,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="62"/>
+      <c r="M8" s="67"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1978,7 +2061,7 @@
       <c r="C10" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="D10" s="63" t="s">
         <v>28</v>
       </c>
       <c r="E10" s="37" t="s">
@@ -2015,7 +2098,7 @@
       <c r="C11" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="64" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="39" t="s">
@@ -2052,7 +2135,7 @@
       <c r="C12" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="36" t="s">
+      <c r="D12" s="63" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="37" t="s">
@@ -2089,7 +2172,7 @@
       <c r="C13" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="64" t="s">
         <v>31</v>
       </c>
       <c r="E13" s="39" t="s">
@@ -2126,7 +2209,7 @@
       <c r="C14" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="36" t="s">
+      <c r="D14" s="63" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="37" t="s">
@@ -2163,7 +2246,7 @@
       <c r="C15" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="64" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="39" t="s">
@@ -2200,7 +2283,7 @@
       <c r="C16" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="63" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="37" t="s">
@@ -2237,7 +2320,7 @@
       <c r="C17" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="64" t="s">
         <v>35</v>
       </c>
       <c r="E17" s="39" t="s">
@@ -2274,7 +2357,7 @@
       <c r="C18" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="36" t="s">
+      <c r="D18" s="63" t="s">
         <v>36</v>
       </c>
       <c r="E18" s="37" t="s">
@@ -2311,7 +2394,7 @@
       <c r="C19" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="64" t="s">
         <v>37</v>
       </c>
       <c r="E19" s="39" t="s">
@@ -2348,7 +2431,7 @@
       <c r="C20" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="36" t="s">
+      <c r="D20" s="63" t="s">
         <v>38</v>
       </c>
       <c r="E20" s="37" t="s">
@@ -2385,7 +2468,7 @@
       <c r="C21" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="64" t="s">
         <v>39</v>
       </c>
       <c r="E21" s="39" t="s">
@@ -2422,7 +2505,7 @@
       <c r="C22" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="63" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="37" t="s">
@@ -2459,7 +2542,7 @@
       <c r="C23" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="64" t="s">
         <v>41</v>
       </c>
       <c r="E23" s="39" t="s">
@@ -2496,7 +2579,7 @@
       <c r="C24" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="36" t="s">
+      <c r="D24" s="63" t="s">
         <v>42</v>
       </c>
       <c r="E24" s="37" t="s">
@@ -2533,7 +2616,7 @@
       <c r="C25" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="64" t="s">
         <v>43</v>
       </c>
       <c r="E25" s="39" t="s">
@@ -2570,7 +2653,7 @@
       <c r="C26" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="D26" s="36" t="s">
+      <c r="D26" s="63" t="s">
         <v>44</v>
       </c>
       <c r="E26" s="37" t="s">
@@ -2607,7 +2690,7 @@
       <c r="C27" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="64" t="s">
         <v>45</v>
       </c>
       <c r="E27" s="39" t="s">
@@ -2644,7 +2727,7 @@
       <c r="C28" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="63" t="s">
         <v>46</v>
       </c>
       <c r="E28" s="37" t="s">
@@ -2781,8 +2864,8 @@
         <f t="shared" ref="L31" si="11">K31*5</f>
         <v>20</v>
       </c>
-      <c r="M31" s="65" t="s">
-        <v>274</v>
+      <c r="M31" s="62" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3238,34 +3321,34 @@
       <c r="C44" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="D44" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="E44" s="64" t="s">
+      <c r="E44" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="F44" s="63" t="s">
+      <c r="F44" s="60" t="s">
         <v>152</v>
       </c>
-      <c r="G44" s="64" t="s">
+      <c r="G44" s="61" t="s">
         <v>195</v>
       </c>
-      <c r="H44" s="63" t="s">
+      <c r="H44" s="60" t="s">
         <v>210</v>
       </c>
-      <c r="I44" s="64" t="s">
+      <c r="I44" s="61" t="s">
         <v>255</v>
       </c>
-      <c r="J44" s="63"/>
-      <c r="K44" s="63">
+      <c r="J44" s="60"/>
+      <c r="K44" s="60">
         <v>2</v>
       </c>
-      <c r="L44" s="64">
+      <c r="L44" s="61">
         <f>K44*5</f>
         <v>10</v>
       </c>
-      <c r="M44" s="65" t="s">
-        <v>274</v>
+      <c r="M44" s="62" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3449,8 +3532,8 @@
         <f t="shared" ref="L49" si="20">K49*5</f>
         <v>50</v>
       </c>
-      <c r="M49" s="65" t="s">
-        <v>274</v>
+      <c r="M49" s="62" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3899,7 +3982,7 @@
       </c>
       <c r="M61" s="36"/>
     </row>
-    <row r="62" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="50">
         <f>ROW(B62) - ROW($B$9)</f>
@@ -3912,7 +3995,7 @@
         <v>268</v>
       </c>
       <c r="E62" s="36" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F62" s="36" t="s">
         <v>265</v>
@@ -3938,35 +4021,72 @@
       </c>
       <c r="M62" s="36"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
-      <c r="B63" s="31"/>
-      <c r="C63" s="48"/>
-      <c r="D63" s="32"/>
-      <c r="E63" s="33"/>
-      <c r="F63" s="34"/>
-      <c r="G63" s="35"/>
-      <c r="H63" s="34"/>
-      <c r="I63" s="35"/>
-      <c r="J63" s="35"/>
-      <c r="K63" s="35"/>
-      <c r="L63" s="35"/>
-      <c r="M63" s="41"/>
-    </row>
-    <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="50">
+        <f>ROW(B63) - ROW($B$9)</f>
+        <v>54</v>
+      </c>
+      <c r="C63" s="55" t="s">
+        <v>275</v>
+      </c>
+      <c r="D63" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="E63" s="36" t="s">
+        <v>277</v>
+      </c>
+      <c r="F63" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="G63" s="36" t="s">
+        <v>276</v>
+      </c>
+      <c r="H63" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="I63" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J63" s="59"/>
+      <c r="K63" s="36">
+        <v>1</v>
+      </c>
+      <c r="L63" s="36">
+        <f>K63*5</f>
+        <v>5</v>
+      </c>
+      <c r="M63" s="36"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="B64" s="24"/>
-      <c r="C64" s="49"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="9"/>
-      <c r="J64" s="9"/>
-      <c r="K64" s="9"/>
-      <c r="L64" s="9"/>
-      <c r="M64" s="42"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="48"/>
+      <c r="D64" s="32"/>
+      <c r="E64" s="33"/>
+      <c r="F64" s="34"/>
+      <c r="G64" s="35"/>
+      <c r="H64" s="34"/>
+      <c r="I64" s="35"/>
+      <c r="J64" s="35"/>
+      <c r="K64" s="35"/>
+      <c r="L64" s="35"/>
+      <c r="M64" s="41"/>
+    </row>
+    <row r="65" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="1"/>
+      <c r="B65" s="24"/>
+      <c r="C65" s="49"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="9"/>
+      <c r="M65" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3981,4 +4101,2248 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
   <drawing r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M65"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="10"/>
+      <c r="F2" s="52" t="s">
+        <v>260</v>
+      </c>
+      <c r="G2" s="11"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="40"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="53" t="s">
+        <v>261</v>
+      </c>
+      <c r="G3" s="12"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="66"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="53" t="s">
+        <v>261</v>
+      </c>
+      <c r="G4" s="13"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="67"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="54" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="14"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="67"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="67"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="67"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="67"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="H9" s="29" t="s">
+        <v>209</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>262</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>269</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="L9" s="51" t="s">
+        <v>263</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="68"/>
+      <c r="B10" s="50">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="H10" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>236</v>
+      </c>
+      <c r="J10" s="36"/>
+      <c r="K10" s="36">
+        <v>6</v>
+      </c>
+      <c r="L10" s="37">
+        <f>K10*5</f>
+        <v>30</v>
+      </c>
+      <c r="M10" s="36"/>
+    </row>
+    <row r="11" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="68"/>
+      <c r="B11" s="50">
+        <f t="shared" ref="B11:B59" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="64" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="G11" s="39" t="s">
+        <v>167</v>
+      </c>
+      <c r="H11" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I11" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="J11" s="38"/>
+      <c r="K11" s="38">
+        <v>15</v>
+      </c>
+      <c r="L11" s="39">
+        <f t="shared" ref="L11" si="1">K11*5</f>
+        <v>75</v>
+      </c>
+      <c r="M11" s="38"/>
+    </row>
+    <row r="12" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="68"/>
+      <c r="B12" s="50">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="H12" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36">
+        <v>4</v>
+      </c>
+      <c r="L12" s="37">
+        <f>K12*5</f>
+        <v>20</v>
+      </c>
+      <c r="M12" s="36"/>
+    </row>
+    <row r="13" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="68"/>
+      <c r="B13" s="50">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="64" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13" s="39" t="s">
+        <v>169</v>
+      </c>
+      <c r="H13" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I13" s="39" t="s">
+        <v>239</v>
+      </c>
+      <c r="J13" s="38"/>
+      <c r="K13" s="38">
+        <v>2</v>
+      </c>
+      <c r="L13" s="39">
+        <f t="shared" ref="L13" si="2">K13*5</f>
+        <v>10</v>
+      </c>
+      <c r="M13" s="38"/>
+    </row>
+    <row r="14" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="68"/>
+      <c r="B14" s="50">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="H14" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>240</v>
+      </c>
+      <c r="J14" s="36"/>
+      <c r="K14" s="36">
+        <v>5</v>
+      </c>
+      <c r="L14" s="37">
+        <f>K14*5</f>
+        <v>25</v>
+      </c>
+      <c r="M14" s="36"/>
+    </row>
+    <row r="15" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="68"/>
+      <c r="B15" s="50">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="64" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="G15" s="39" t="s">
+        <v>171</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I15" s="39" t="s">
+        <v>241</v>
+      </c>
+      <c r="J15" s="38"/>
+      <c r="K15" s="38">
+        <v>4</v>
+      </c>
+      <c r="L15" s="39">
+        <f t="shared" ref="L15" si="3">K15*5</f>
+        <v>20</v>
+      </c>
+      <c r="M15" s="38"/>
+    </row>
+    <row r="16" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="68"/>
+      <c r="B16" s="50">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="63" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="F16" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="H16" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>242</v>
+      </c>
+      <c r="J16" s="36"/>
+      <c r="K16" s="36">
+        <v>1</v>
+      </c>
+      <c r="L16" s="37">
+        <f>K16*5</f>
+        <v>5</v>
+      </c>
+      <c r="M16" s="36"/>
+    </row>
+    <row r="17" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="68"/>
+      <c r="B17" s="50">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="64" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="G17" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="H17" s="38" t="s">
+        <v>211</v>
+      </c>
+      <c r="I17" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J17" s="38"/>
+      <c r="K17" s="38">
+        <v>1</v>
+      </c>
+      <c r="L17" s="39">
+        <f t="shared" ref="L17" si="4">K17*5</f>
+        <v>5</v>
+      </c>
+      <c r="M17" s="38"/>
+    </row>
+    <row r="18" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="68"/>
+      <c r="B18" s="50">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="63" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="H18" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J18" s="36"/>
+      <c r="K18" s="36">
+        <v>1</v>
+      </c>
+      <c r="L18" s="37">
+        <f>K18*5</f>
+        <v>5</v>
+      </c>
+      <c r="M18" s="36"/>
+    </row>
+    <row r="19" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="68"/>
+      <c r="B19" s="50">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="G19" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>213</v>
+      </c>
+      <c r="I19" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J19" s="38"/>
+      <c r="K19" s="38">
+        <v>1</v>
+      </c>
+      <c r="L19" s="39">
+        <f t="shared" ref="L19" si="5">K19*5</f>
+        <v>5</v>
+      </c>
+      <c r="M19" s="38"/>
+    </row>
+    <row r="20" spans="1:13" s="69" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="68"/>
+      <c r="B20" s="50">
+        <f>ROW(B20) - ROW($B$9)</f>
+        <v>11</v>
+      </c>
+      <c r="C20" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="63" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="G20" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="H20" s="36" t="s">
+        <v>214</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36">
+        <v>3</v>
+      </c>
+      <c r="L20" s="37">
+        <f>K20*5</f>
+        <v>15</v>
+      </c>
+      <c r="M20" s="36"/>
+    </row>
+    <row r="21" spans="1:13" s="69" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="68"/>
+      <c r="B21" s="50">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="G21" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="H21" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="I21" s="39" t="s">
+        <v>243</v>
+      </c>
+      <c r="J21" s="38"/>
+      <c r="K21" s="38">
+        <v>1</v>
+      </c>
+      <c r="L21" s="39">
+        <f t="shared" ref="L21" si="6">K21*5</f>
+        <v>5</v>
+      </c>
+      <c r="M21" s="38"/>
+    </row>
+    <row r="22" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="68"/>
+      <c r="B22" s="50">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="63" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="H22" s="36" t="s">
+        <v>215</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J22" s="36"/>
+      <c r="K22" s="36">
+        <v>1</v>
+      </c>
+      <c r="L22" s="37">
+        <f>K22*5</f>
+        <v>5</v>
+      </c>
+      <c r="M22" s="36"/>
+    </row>
+    <row r="23" spans="1:13" s="69" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="68"/>
+      <c r="B23" s="50">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="64" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="G23" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="H23" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="I23" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J23" s="38"/>
+      <c r="K23" s="38">
+        <v>1</v>
+      </c>
+      <c r="L23" s="39">
+        <f t="shared" ref="L23" si="7">K23*5</f>
+        <v>5</v>
+      </c>
+      <c r="M23" s="38"/>
+    </row>
+    <row r="24" spans="1:13" s="69" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="68"/>
+      <c r="B24" s="50">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="63" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="H24" s="36" t="s">
+        <v>217</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J24" s="36"/>
+      <c r="K24" s="36">
+        <v>1</v>
+      </c>
+      <c r="L24" s="37">
+        <f>K24*5</f>
+        <v>5</v>
+      </c>
+      <c r="M24" s="36"/>
+    </row>
+    <row r="25" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="68"/>
+      <c r="B25" s="50">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="64" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="G25" s="39">
+        <v>61300211121</v>
+      </c>
+      <c r="H25" s="38" t="s">
+        <v>218</v>
+      </c>
+      <c r="I25" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J25" s="38"/>
+      <c r="K25" s="38">
+        <v>1</v>
+      </c>
+      <c r="L25" s="39">
+        <f t="shared" ref="L25" si="8">K25*5</f>
+        <v>5</v>
+      </c>
+      <c r="M25" s="38"/>
+    </row>
+    <row r="26" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="68"/>
+      <c r="B26" s="50">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="63" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="H26" s="36" t="s">
+        <v>219</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="J26" s="36"/>
+      <c r="K26" s="36">
+        <v>1</v>
+      </c>
+      <c r="L26" s="37">
+        <f>K26*5</f>
+        <v>5</v>
+      </c>
+      <c r="M26" s="36"/>
+    </row>
+    <row r="27" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="68"/>
+      <c r="B27" s="50">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="64" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="G27" s="39" t="s">
+        <v>146</v>
+      </c>
+      <c r="H27" s="38" t="s">
+        <v>220</v>
+      </c>
+      <c r="I27" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="J27" s="38"/>
+      <c r="K27" s="38">
+        <v>2</v>
+      </c>
+      <c r="L27" s="39">
+        <f t="shared" ref="L27" si="9">K27*5</f>
+        <v>10</v>
+      </c>
+      <c r="M27" s="38"/>
+    </row>
+    <row r="28" spans="1:13" s="69" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="68"/>
+      <c r="B28" s="50">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="55" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="63" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="F28" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J28" s="36"/>
+      <c r="K28" s="36">
+        <v>1</v>
+      </c>
+      <c r="L28" s="37">
+        <f>K28*5</f>
+        <v>5</v>
+      </c>
+      <c r="M28" s="36"/>
+    </row>
+    <row r="29" spans="1:13" s="69" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="68"/>
+      <c r="B29" s="50">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C29" s="55" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="G29" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="H29" s="38" t="s">
+        <v>221</v>
+      </c>
+      <c r="I29" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J29" s="38"/>
+      <c r="K29" s="38">
+        <v>1</v>
+      </c>
+      <c r="L29" s="39">
+        <f t="shared" ref="L29" si="10">K29*5</f>
+        <v>5</v>
+      </c>
+      <c r="M29" s="38"/>
+    </row>
+    <row r="30" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="68"/>
+      <c r="B30" s="50">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="H30" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J30" s="36"/>
+      <c r="K30" s="36">
+        <v>3</v>
+      </c>
+      <c r="L30" s="37">
+        <f>K30*5</f>
+        <v>15</v>
+      </c>
+      <c r="M30" s="36"/>
+    </row>
+    <row r="31" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="68"/>
+      <c r="B31" s="50">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="57" t="s">
+        <v>49</v>
+      </c>
+      <c r="E31" s="58" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="G31" s="58" t="s">
+        <v>265</v>
+      </c>
+      <c r="H31" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="I31" s="58" t="s">
+        <v>265</v>
+      </c>
+      <c r="J31" s="57"/>
+      <c r="K31" s="57">
+        <v>4</v>
+      </c>
+      <c r="L31" s="58">
+        <f t="shared" ref="L31" si="11">K31*5</f>
+        <v>20</v>
+      </c>
+      <c r="M31" s="62" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" s="69" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="68"/>
+      <c r="B32" s="50">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>149</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="H32" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J32" s="36"/>
+      <c r="K32" s="36">
+        <v>2</v>
+      </c>
+      <c r="L32" s="37">
+        <f>K32*5</f>
+        <v>10</v>
+      </c>
+      <c r="M32" s="36"/>
+    </row>
+    <row r="33" spans="1:13" s="69" customFormat="1" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="68"/>
+      <c r="B33" s="50">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C33" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="G33" s="39" t="s">
+        <v>184</v>
+      </c>
+      <c r="H33" s="38" t="s">
+        <v>224</v>
+      </c>
+      <c r="I33" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J33" s="38"/>
+      <c r="K33" s="38">
+        <v>3</v>
+      </c>
+      <c r="L33" s="39">
+        <f t="shared" ref="L33" si="12">K33*5</f>
+        <v>15</v>
+      </c>
+      <c r="M33" s="38"/>
+    </row>
+    <row r="34" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="68"/>
+      <c r="B34" s="50">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="F34" s="36" t="s">
+        <v>151</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="H34" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J34" s="36"/>
+      <c r="K34" s="36">
+        <v>1</v>
+      </c>
+      <c r="L34" s="37">
+        <f>K34*5</f>
+        <v>5</v>
+      </c>
+      <c r="M34" s="36"/>
+    </row>
+    <row r="35" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="68"/>
+      <c r="B35" s="50">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C35" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="F35" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G35" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="H35" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I35" s="39" t="s">
+        <v>246</v>
+      </c>
+      <c r="J35" s="38"/>
+      <c r="K35" s="38">
+        <v>2</v>
+      </c>
+      <c r="L35" s="39">
+        <f t="shared" ref="L35" si="13">K35*5</f>
+        <v>10</v>
+      </c>
+      <c r="M35" s="38"/>
+    </row>
+    <row r="36" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="68"/>
+      <c r="B36" s="50">
+        <f>ROW(B36) - ROW($B$9)</f>
+        <v>27</v>
+      </c>
+      <c r="C36" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="F36" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="H36" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>247</v>
+      </c>
+      <c r="J36" s="36"/>
+      <c r="K36" s="36">
+        <v>1</v>
+      </c>
+      <c r="L36" s="37">
+        <f>K36*5</f>
+        <v>5</v>
+      </c>
+      <c r="M36" s="36"/>
+    </row>
+    <row r="37" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="68"/>
+      <c r="B37" s="50">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C37" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E37" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="F37" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G37" s="39" t="s">
+        <v>188</v>
+      </c>
+      <c r="H37" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I37" s="39" t="s">
+        <v>248</v>
+      </c>
+      <c r="J37" s="38"/>
+      <c r="K37" s="38">
+        <v>1</v>
+      </c>
+      <c r="L37" s="39">
+        <f t="shared" ref="L37" si="14">K37*5</f>
+        <v>5</v>
+      </c>
+      <c r="M37" s="38"/>
+    </row>
+    <row r="38" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="68"/>
+      <c r="B38" s="50">
+        <f>ROW(B38) - ROW($B$9)</f>
+        <v>29</v>
+      </c>
+      <c r="C38" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="F38" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="G38" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="H38" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="I38" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="J38" s="36"/>
+      <c r="K38" s="36">
+        <v>1</v>
+      </c>
+      <c r="L38" s="37">
+        <f>K38*5</f>
+        <v>5</v>
+      </c>
+      <c r="M38" s="36"/>
+    </row>
+    <row r="39" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="68"/>
+      <c r="B39" s="50">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="C39" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F39" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G39" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="H39" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I39" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="J39" s="38"/>
+      <c r="K39" s="38">
+        <v>8</v>
+      </c>
+      <c r="L39" s="39">
+        <f t="shared" ref="L39" si="15">K39*5</f>
+        <v>40</v>
+      </c>
+      <c r="M39" s="38"/>
+    </row>
+    <row r="40" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="68"/>
+      <c r="B40" s="50">
+        <f>ROW(B40) - ROW($B$9)</f>
+        <v>31</v>
+      </c>
+      <c r="C40" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F40" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="G40" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="H40" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="I40" s="37" t="s">
+        <v>251</v>
+      </c>
+      <c r="J40" s="36"/>
+      <c r="K40" s="36">
+        <v>1</v>
+      </c>
+      <c r="L40" s="37">
+        <f>K40*5</f>
+        <v>5</v>
+      </c>
+      <c r="M40" s="36"/>
+    </row>
+    <row r="41" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="68"/>
+      <c r="B41" s="50">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C41" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E41" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="F41" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G41" s="39" t="s">
+        <v>192</v>
+      </c>
+      <c r="H41" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I41" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="J41" s="38"/>
+      <c r="K41" s="38">
+        <v>3</v>
+      </c>
+      <c r="L41" s="39">
+        <f t="shared" ref="L41" si="16">K41*5</f>
+        <v>15</v>
+      </c>
+      <c r="M41" s="38"/>
+    </row>
+    <row r="42" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="68"/>
+      <c r="B42" s="50">
+        <f>ROW(B42) - ROW($B$9)</f>
+        <v>33</v>
+      </c>
+      <c r="C42" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="E42" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="F42" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="G42" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="H42" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I42" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="J42" s="36"/>
+      <c r="K42" s="36">
+        <v>3</v>
+      </c>
+      <c r="L42" s="37">
+        <f>K42*5</f>
+        <v>15</v>
+      </c>
+      <c r="M42" s="36"/>
+    </row>
+    <row r="43" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="68"/>
+      <c r="B43" s="50">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="C43" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E43" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="F43" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G43" s="39" t="s">
+        <v>194</v>
+      </c>
+      <c r="H43" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I43" s="39" t="s">
+        <v>254</v>
+      </c>
+      <c r="J43" s="38"/>
+      <c r="K43" s="38">
+        <v>2</v>
+      </c>
+      <c r="L43" s="39">
+        <f t="shared" ref="L43" si="17">K43*5</f>
+        <v>10</v>
+      </c>
+      <c r="M43" s="38"/>
+    </row>
+    <row r="44" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="68"/>
+      <c r="B44" s="50">
+        <f>ROW(B44) - ROW($B$9)</f>
+        <v>35</v>
+      </c>
+      <c r="C44" s="56" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="60" t="s">
+        <v>62</v>
+      </c>
+      <c r="E44" s="61" t="s">
+        <v>114</v>
+      </c>
+      <c r="F44" s="60" t="s">
+        <v>152</v>
+      </c>
+      <c r="G44" s="61" t="s">
+        <v>195</v>
+      </c>
+      <c r="H44" s="60" t="s">
+        <v>210</v>
+      </c>
+      <c r="I44" s="61" t="s">
+        <v>255</v>
+      </c>
+      <c r="J44" s="60"/>
+      <c r="K44" s="60">
+        <v>2</v>
+      </c>
+      <c r="L44" s="61">
+        <f>K44*5</f>
+        <v>10</v>
+      </c>
+      <c r="M44" s="62" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="68"/>
+      <c r="B45" s="50">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="C45" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="F45" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="G45" s="39" t="s">
+        <v>196</v>
+      </c>
+      <c r="H45" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I45" s="39" t="s">
+        <v>256</v>
+      </c>
+      <c r="J45" s="38"/>
+      <c r="K45" s="38">
+        <v>4</v>
+      </c>
+      <c r="L45" s="39">
+        <f t="shared" ref="L45" si="18">K45*5</f>
+        <v>20</v>
+      </c>
+      <c r="M45" s="38"/>
+    </row>
+    <row r="46" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="68"/>
+      <c r="B46" s="50">
+        <f>ROW(B46) - ROW($B$9)</f>
+        <v>37</v>
+      </c>
+      <c r="C46" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="36" t="s">
+        <v>64</v>
+      </c>
+      <c r="E46" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="F46" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="G46" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="H46" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="I46" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="J46" s="36"/>
+      <c r="K46" s="36">
+        <v>4</v>
+      </c>
+      <c r="L46" s="37">
+        <f>K46*5</f>
+        <v>20</v>
+      </c>
+      <c r="M46" s="36"/>
+    </row>
+    <row r="47" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="68"/>
+      <c r="B47" s="50">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="C47" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="E47" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="F47" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="G47" s="39" t="s">
+        <v>198</v>
+      </c>
+      <c r="H47" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I47" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="J47" s="38"/>
+      <c r="K47" s="38">
+        <v>2</v>
+      </c>
+      <c r="L47" s="39">
+        <f t="shared" ref="L47" si="19">K47*5</f>
+        <v>10</v>
+      </c>
+      <c r="M47" s="38"/>
+    </row>
+    <row r="48" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="68"/>
+      <c r="B48" s="50">
+        <f>ROW(B48) - ROW($B$9)</f>
+        <v>39</v>
+      </c>
+      <c r="C48" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="E48" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="F48" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="G48" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="H48" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="I48" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="J48" s="36"/>
+      <c r="K48" s="36">
+        <v>1</v>
+      </c>
+      <c r="L48" s="37">
+        <f>K48*5</f>
+        <v>5</v>
+      </c>
+      <c r="M48" s="36"/>
+    </row>
+    <row r="49" spans="1:13" s="69" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="68"/>
+      <c r="B49" s="50">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="C49" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="D49" s="57" t="s">
+        <v>67</v>
+      </c>
+      <c r="E49" s="58" t="s">
+        <v>119</v>
+      </c>
+      <c r="F49" s="57" t="s">
+        <v>266</v>
+      </c>
+      <c r="G49" s="58" t="s">
+        <v>22</v>
+      </c>
+      <c r="H49" s="57"/>
+      <c r="I49" s="58" t="s">
+        <v>265</v>
+      </c>
+      <c r="J49" s="57"/>
+      <c r="K49" s="57">
+        <v>10</v>
+      </c>
+      <c r="L49" s="58">
+        <f t="shared" ref="L49" si="20">K49*5</f>
+        <v>50</v>
+      </c>
+      <c r="M49" s="62" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" s="69" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="68"/>
+      <c r="B50" s="50">
+        <f>ROW(B50) - ROW($B$9)</f>
+        <v>41</v>
+      </c>
+      <c r="C50" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="D50" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="E50" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="F50" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="G50" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="H50" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="I50" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J50" s="36"/>
+      <c r="K50" s="36">
+        <v>1</v>
+      </c>
+      <c r="L50" s="37">
+        <f>K50*5</f>
+        <v>5</v>
+      </c>
+      <c r="M50" s="36"/>
+    </row>
+    <row r="51" spans="1:13" s="69" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="68"/>
+      <c r="B51" s="50">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C51" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D51" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="E51" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="F51" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="G51" s="39" t="s">
+        <v>155</v>
+      </c>
+      <c r="H51" s="38" t="s">
+        <v>229</v>
+      </c>
+      <c r="I51" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J51" s="38"/>
+      <c r="K51" s="38">
+        <v>4</v>
+      </c>
+      <c r="L51" s="39">
+        <f t="shared" ref="L51" si="21">K51*5</f>
+        <v>20</v>
+      </c>
+      <c r="M51" s="38"/>
+    </row>
+    <row r="52" spans="1:13" s="69" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="68"/>
+      <c r="B52" s="50">
+        <f>ROW(B52) - ROW($B$9)</f>
+        <v>43</v>
+      </c>
+      <c r="C52" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="D52" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E52" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="F52" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="G52" s="37" t="s">
+        <v>200</v>
+      </c>
+      <c r="H52" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="I52" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J52" s="36"/>
+      <c r="K52" s="36">
+        <v>1</v>
+      </c>
+      <c r="L52" s="37">
+        <f>K52*5</f>
+        <v>5</v>
+      </c>
+      <c r="M52" s="36"/>
+    </row>
+    <row r="53" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="68"/>
+      <c r="B53" s="50">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C53" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="38" t="s">
+        <v>71</v>
+      </c>
+      <c r="E53" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="F53" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="G53" s="39" t="s">
+        <v>201</v>
+      </c>
+      <c r="H53" s="38" t="s">
+        <v>230</v>
+      </c>
+      <c r="I53" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J53" s="38"/>
+      <c r="K53" s="38">
+        <v>1</v>
+      </c>
+      <c r="L53" s="39">
+        <f t="shared" ref="L53" si="22">K53*5</f>
+        <v>5</v>
+      </c>
+      <c r="M53" s="38"/>
+    </row>
+    <row r="54" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="68"/>
+      <c r="B54" s="50">
+        <f>ROW(B54) - ROW($B$9)</f>
+        <v>45</v>
+      </c>
+      <c r="C54" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D54" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="E54" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="F54" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="G54" s="37" t="s">
+        <v>202</v>
+      </c>
+      <c r="H54" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="I54" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J54" s="36"/>
+      <c r="K54" s="36">
+        <v>1</v>
+      </c>
+      <c r="L54" s="37">
+        <f>K54*5</f>
+        <v>5</v>
+      </c>
+      <c r="M54" s="36"/>
+    </row>
+    <row r="55" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="68"/>
+      <c r="B55" s="50">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="C55" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D55" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="F55" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="G55" s="39" t="s">
+        <v>203</v>
+      </c>
+      <c r="H55" s="38" t="s">
+        <v>231</v>
+      </c>
+      <c r="I55" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J55" s="38"/>
+      <c r="K55" s="38">
+        <v>1</v>
+      </c>
+      <c r="L55" s="39">
+        <f t="shared" ref="L55" si="23">K55*5</f>
+        <v>5</v>
+      </c>
+      <c r="M55" s="38"/>
+    </row>
+    <row r="56" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="68"/>
+      <c r="B56" s="50">
+        <f>ROW(B56) - ROW($B$9)</f>
+        <v>47</v>
+      </c>
+      <c r="C56" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="D56" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="E56" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="F56" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="G56" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="H56" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="I56" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J56" s="36"/>
+      <c r="K56" s="36">
+        <v>1</v>
+      </c>
+      <c r="L56" s="37">
+        <f>K56*5</f>
+        <v>5</v>
+      </c>
+      <c r="M56" s="36"/>
+    </row>
+    <row r="57" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="68"/>
+      <c r="B57" s="50">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="C57" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D57" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="E57" s="39" t="s">
+        <v>127</v>
+      </c>
+      <c r="F57" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="G57" s="39" t="s">
+        <v>205</v>
+      </c>
+      <c r="H57" s="38" t="s">
+        <v>233</v>
+      </c>
+      <c r="I57" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J57" s="38"/>
+      <c r="K57" s="38">
+        <v>1</v>
+      </c>
+      <c r="L57" s="39">
+        <f t="shared" ref="L57" si="24">K57*5</f>
+        <v>5</v>
+      </c>
+      <c r="M57" s="38"/>
+    </row>
+    <row r="58" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="68"/>
+      <c r="B58" s="50">
+        <f>ROW(B58) - ROW($B$9)</f>
+        <v>49</v>
+      </c>
+      <c r="C58" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D58" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="E58" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="F58" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="G58" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="H58" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="I58" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J58" s="36"/>
+      <c r="K58" s="36">
+        <v>1</v>
+      </c>
+      <c r="L58" s="37">
+        <f>K58*5</f>
+        <v>5</v>
+      </c>
+      <c r="M58" s="36"/>
+    </row>
+    <row r="59" spans="1:13" s="69" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="68"/>
+      <c r="B59" s="50">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="C59" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D59" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="E59" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="F59" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="G59" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="H59" s="38" t="s">
+        <v>235</v>
+      </c>
+      <c r="I59" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J59" s="38"/>
+      <c r="K59" s="38">
+        <v>1</v>
+      </c>
+      <c r="L59" s="39">
+        <f t="shared" ref="L59" si="25">K59*5</f>
+        <v>5</v>
+      </c>
+      <c r="M59" s="38"/>
+    </row>
+    <row r="60" spans="1:13" s="69" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="68"/>
+      <c r="B60" s="50">
+        <f>ROW(B60) - ROW($B$9)</f>
+        <v>51</v>
+      </c>
+      <c r="C60" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D60" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E60" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="F60" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="G60" s="37" t="s">
+        <v>208</v>
+      </c>
+      <c r="H60" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="I60" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="J60" s="36"/>
+      <c r="K60" s="36">
+        <v>1</v>
+      </c>
+      <c r="L60" s="37">
+        <f>K60*5</f>
+        <v>5</v>
+      </c>
+      <c r="M60" s="36"/>
+    </row>
+    <row r="61" spans="1:13" s="69" customFormat="1" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="68"/>
+      <c r="B61" s="50">
+        <f>ROW(B61) - ROW($B$9)</f>
+        <v>52</v>
+      </c>
+      <c r="C61" s="55" t="s">
+        <v>267</v>
+      </c>
+      <c r="D61" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="E61" s="36" t="s">
+        <v>271</v>
+      </c>
+      <c r="F61" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="G61" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="H61" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="I61" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J61" s="59" t="s">
+        <v>270</v>
+      </c>
+      <c r="K61" s="36">
+        <v>1</v>
+      </c>
+      <c r="L61" s="36">
+        <f>K61*5</f>
+        <v>5</v>
+      </c>
+      <c r="M61" s="36"/>
+    </row>
+    <row r="62" spans="1:13" s="69" customFormat="1" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="68"/>
+      <c r="B62" s="50">
+        <f>ROW(B62) - ROW($B$9)</f>
+        <v>53</v>
+      </c>
+      <c r="C62" s="55" t="s">
+        <v>272</v>
+      </c>
+      <c r="D62" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="E62" s="36" t="s">
+        <v>274</v>
+      </c>
+      <c r="F62" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="G62" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="H62" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="I62" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J62" s="59" t="s">
+        <v>270</v>
+      </c>
+      <c r="K62" s="36">
+        <v>1</v>
+      </c>
+      <c r="L62" s="36">
+        <f>K62*5</f>
+        <v>5</v>
+      </c>
+      <c r="M62" s="36"/>
+    </row>
+    <row r="63" spans="1:13" s="69" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="68"/>
+      <c r="B63" s="50">
+        <f>ROW(B63) - ROW($B$9)</f>
+        <v>54</v>
+      </c>
+      <c r="C63" s="55" t="s">
+        <v>275</v>
+      </c>
+      <c r="D63" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="E63" s="36" t="s">
+        <v>277</v>
+      </c>
+      <c r="F63" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="G63" s="36" t="s">
+        <v>276</v>
+      </c>
+      <c r="H63" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="I63" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="J63" s="59"/>
+      <c r="K63" s="36">
+        <v>1</v>
+      </c>
+      <c r="L63" s="36">
+        <f>K63*5</f>
+        <v>5</v>
+      </c>
+      <c r="M63" s="36"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" s="1"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="48"/>
+      <c r="D64" s="32"/>
+      <c r="E64" s="33"/>
+      <c r="F64" s="34"/>
+      <c r="G64" s="35"/>
+      <c r="H64" s="34"/>
+      <c r="I64" s="35"/>
+      <c r="J64" s="35"/>
+      <c r="K64" s="35"/>
+      <c r="L64" s="35"/>
+      <c r="M64" s="41"/>
+    </row>
+    <row r="65" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="1"/>
+      <c r="B65" s="24"/>
+      <c r="C65" s="49"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="9"/>
+      <c r="M65" s="42"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="I1:M1"/>
+    <mergeCell ref="M3:M8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="J61" r:id="rId1"/>
+    <hyperlink ref="J62" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>